<commit_message>
Add 2026 PSI Annual Conference poster
</commit_message>
<xml_diff>
--- a/data/seminars.xlsx
+++ b/data/seminars.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="110" documentId="13_ncr:1_{AE9F6201-8E07-4B78-AE68-6B047CA8E52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8D2579B-45A1-423E-BBBC-0A96C0DBA5DD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FDEE638-9262-4F47-8435-88ADEBF9A500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="18000" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191028" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="140">
   <si>
     <t>date</t>
   </si>
@@ -81,356 +81,383 @@
     <t>link</t>
   </si>
   <si>
+    <t>12.06.2022</t>
+  </si>
+  <si>
+    <t>2022 PSI Annual Conference</t>
+  </si>
+  <si>
+    <t>https://www.psiweb.org/events/event-item/2022/06/12/default-calendar/2022-psi-annual-conference</t>
+  </si>
+  <si>
+    <t>Gothenburg</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>F2F</t>
+  </si>
+  <si>
+    <t>Poster</t>
+  </si>
+  <si>
+    <t>Stefan Englert</t>
+  </si>
+  <si>
+    <t>J&amp;J</t>
+  </si>
+  <si>
+    <t>UPDATE - Estimand Implementation Working Group (EIWG)</t>
+  </si>
+  <si>
+    <t>EIWG-PSI-2022-Poster.pdf</t>
+  </si>
+  <si>
+    <t>Helle Lynggaard</t>
+  </si>
+  <si>
+    <t>Novo Nordisk</t>
+  </si>
+  <si>
+    <t>Does the Estimand Framework Add Value to Clinical Pharmacology Trials?</t>
+  </si>
+  <si>
+    <t>EIWG_Clinical_Pharmacology_PSI_poster_02June2022_handout.pdf</t>
+  </si>
+  <si>
+    <t>01.11.2022</t>
+  </si>
+  <si>
+    <t>EFSPI Newsletter</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t>Article</t>
+  </si>
+  <si>
+    <t>EIWG</t>
+  </si>
+  <si>
+    <t>EIWG brings together statisticians and clinicians to support the estimand journey</t>
+  </si>
+  <si>
+    <t>EFSPI-Christmas-Newsletter-EIWG.pdf</t>
+  </si>
+  <si>
+    <t>13.09.2023</t>
+  </si>
+  <si>
+    <t>8th EFSPI Workshop on Regulatory Statistics 2023</t>
+  </si>
+  <si>
+    <t>Basel</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>How the Estimand Implementation Working Group brings together statisticians and clinicians to support the estimand journey</t>
+  </si>
+  <si>
+    <t>EIWG-EFSPI-Workshop-2023-Poster.pdf</t>
+  </si>
+  <si>
+    <t>11.09.2024</t>
+  </si>
+  <si>
+    <t>2024 EFSPI regulatory statistics workshop</t>
+  </si>
+  <si>
+    <t>Biozentrum Basel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stefan Englert </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> An Appraisal of the ICH E9(R1) Intercurrent Event Definition with Case Examples</t>
+  </si>
+  <si>
+    <t>EIWG-Intercurrent-Events-Poster-Clean.pdf</t>
+  </si>
+  <si>
+    <t>Sue McKendrick</t>
+  </si>
+  <si>
+    <t>PPD Clinical Research Services</t>
+  </si>
+  <si>
+    <t>Considerations when Selecting Strategies for Intercurrent Events in Non-inferiority Trials</t>
+  </si>
+  <si>
+    <t>non-inferiority _poster_final.pdf</t>
+  </si>
+  <si>
+    <t>Vivian Lanius</t>
+  </si>
+  <si>
+    <t>Bayer AG</t>
+  </si>
+  <si>
+    <t>Realizing the benefits of estimands when reporting and communicating study results – some recommendations</t>
+  </si>
+  <si>
+    <t>Poster_EFSPI_EIWG_reporting_2024_final.pdf</t>
+  </si>
+  <si>
+    <t>21.06.2021</t>
+  </si>
+  <si>
+    <t>2021 PSI Annual Conference</t>
+  </si>
+  <si>
+    <t>Virtual</t>
+  </si>
+  <si>
+    <t>Oral presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pepa Polavieja </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lilly </t>
+  </si>
+  <si>
+    <t>ICH E9(R1) Implementation in Study Protocols - Speaker 1</t>
+  </si>
+  <si>
+    <t>PSI presentation_2021.pdf</t>
+  </si>
+  <si>
+    <t>ICH E9(R1) Implementation in Study Protocols - Speaker 2</t>
+  </si>
+  <si>
+    <t>11.06.2023</t>
+  </si>
+  <si>
+    <t>2023 PSI Annual Conference</t>
+  </si>
+  <si>
+    <t>London</t>
+  </si>
+  <si>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>Sunita Rehal</t>
+  </si>
+  <si>
+    <t>GSK</t>
+  </si>
+  <si>
+    <t>The estimands framework in non-inferiority trials:​ Past, Present &amp; Future​</t>
+  </si>
+  <si>
+    <t>12.06.23_13.30-15.00_2_ICH E9(R1)_noninferiority.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paul Terrill </t>
+  </si>
+  <si>
+    <t>Ptstat.co.uk</t>
+  </si>
+  <si>
+    <t>EIWG PSI poster 2022_Final.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helle Lynggaard </t>
+  </si>
+  <si>
+    <t>Does it Make Sense to Apply the Estimand Framework to Clinical Pharmacology Trials? - Speaker 1</t>
+  </si>
+  <si>
+    <t>12.06.23_13.30-15.00_1_ICH E9(R1)_impacts_beyond_Bioequivalence_Sue_Helle.pdf</t>
+  </si>
+  <si>
+    <t>Does it Make Sense to Apply the Estimand Framework to Clinical Pharmacology Trials? - Speaker 2</t>
+  </si>
+  <si>
+    <t>16.06.2024</t>
+  </si>
+  <si>
+    <t>2024 PSI Annual Conference - Talks</t>
+  </si>
+  <si>
+    <t>Amsterdam</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>Non-inferiority and the estimand framework</t>
+  </si>
+  <si>
+    <t>19.06.24_11.00-12.30_Helle_Lynggaard.pdf</t>
+  </si>
+  <si>
+    <t>David Wright</t>
+  </si>
+  <si>
+    <t>AstraZeneca</t>
+  </si>
+  <si>
+    <t>How the estimand framework affects choice of non-inferiority margin</t>
+  </si>
+  <si>
+    <t>19.06.24_11.00-12.30_David_Wright.pdf</t>
+  </si>
+  <si>
+    <t>17.06.2024</t>
+  </si>
+  <si>
+    <t>2024 PSI Annual Conference - Panel</t>
+  </si>
+  <si>
+    <t>Panel discussion</t>
+  </si>
+  <si>
+    <t>Kit Roes</t>
+  </si>
+  <si>
+    <t>Chair EMA MWP</t>
+  </si>
+  <si>
+    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 1</t>
+  </si>
+  <si>
+    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tobias Mütze </t>
+  </si>
+  <si>
     <t>Novartis</t>
   </si>
   <si>
-    <t>AstraZeneca</t>
+    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 3</t>
+  </si>
+  <si>
+    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 4</t>
+  </si>
+  <si>
+    <t>Florian Lasch</t>
   </si>
   <si>
     <t>EMA</t>
   </si>
   <si>
-    <t>London</t>
-  </si>
-  <si>
-    <t>Basel</t>
-  </si>
-  <si>
-    <t>Switzerland</t>
-  </si>
-  <si>
-    <t>Poster</t>
-  </si>
-  <si>
-    <t>Stefan Englert</t>
-  </si>
-  <si>
-    <t>Virtual</t>
-  </si>
-  <si>
-    <t>12.06.2022</t>
-  </si>
-  <si>
-    <t>Gothenburg</t>
-  </si>
-  <si>
-    <t>Sweden</t>
-  </si>
-  <si>
-    <t>F2F</t>
-  </si>
-  <si>
-    <t>J&amp;J</t>
-  </si>
-  <si>
-    <t>GSK</t>
-  </si>
-  <si>
-    <t>Panel discussion</t>
-  </si>
-  <si>
-    <t>David Wright</t>
-  </si>
-  <si>
-    <t>Amsterdam</t>
-  </si>
-  <si>
-    <t>Netherlands</t>
-  </si>
-  <si>
-    <t>UPDATE - Estimand Implementation Working Group (EIWG)</t>
-  </si>
-  <si>
-    <t>EIWG-PSI-2022-Poster.pdf</t>
-  </si>
-  <si>
-    <t>01.11.2022</t>
-  </si>
-  <si>
-    <t>EFSPI Newsletter</t>
-  </si>
-  <si>
-    <t>How the Estimand Implementation Working Group brings together statisticians and clinicians to support the estimand journey</t>
-  </si>
-  <si>
-    <t>EIWG brings together statisticians and clinicians to support the estimand journey</t>
-  </si>
-  <si>
-    <t>13.09.2023</t>
-  </si>
-  <si>
-    <t>2022 PSI Annual Conference</t>
-  </si>
-  <si>
-    <t>Does the Estimand Framework Add Value to Clinical Pharmacology Trials?</t>
-  </si>
-  <si>
-    <t>Helle Lynggaard</t>
-  </si>
-  <si>
-    <t>Sue McKendrick</t>
-  </si>
-  <si>
-    <t>Novo Nordisk</t>
-  </si>
-  <si>
-    <t>PPD Clinical Research Services</t>
+    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khadija Rantell </t>
   </si>
   <si>
     <t>MHRA</t>
   </si>
   <si>
-    <t>2024 EFSPI regulatory statistics workshop</t>
-  </si>
-  <si>
-    <t>Biozentrum Basel</t>
-  </si>
-  <si>
-    <t>11.09.2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stefan Englert </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> An Appraisal of the ICH E9(R1) Intercurrent Event Definition with Case Examples</t>
-  </si>
-  <si>
-    <t>Online</t>
-  </si>
-  <si>
-    <t>8th EFSPI Workshop on Regulatory Statistics 2023</t>
-  </si>
-  <si>
-    <t>Article</t>
-  </si>
-  <si>
-    <t>EIWG</t>
-  </si>
-  <si>
-    <t>EFSPI-Christmas-Newsletter-EIWG.pdf</t>
-  </si>
-  <si>
-    <t>EIWG-EFSPI-Workshop-2023-Poster.pdf</t>
-  </si>
-  <si>
-    <t>2021 PSI Annual Conference</t>
-  </si>
-  <si>
-    <t>Oral presentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pepa Polavieja </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lilly </t>
-  </si>
-  <si>
-    <t>11.06.2023</t>
-  </si>
-  <si>
-    <t>21.06.2021</t>
-  </si>
-  <si>
-    <t>2023 PSI Annual Conference</t>
-  </si>
-  <si>
-    <t>United Kingdom</t>
-  </si>
-  <si>
-    <t>Sunita Rehal</t>
-  </si>
-  <si>
-    <t>The estimands framework in non-inferiority trials:​ Past, Present &amp; Future​</t>
-  </si>
-  <si>
-    <t>12.06.23_13.30-15.00_2_ICH E9(R1)_noninferiority.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paul Terrill </t>
-  </si>
-  <si>
-    <t>Ptstat.co.uk</t>
-  </si>
-  <si>
-    <t>EIWG PSI poster 2022_Final.pdf</t>
-  </si>
-  <si>
-    <t>https://www.psiweb.org/events/event-item/2022/06/12/default-calendar/2022-psi-annual-conference</t>
-  </si>
-  <si>
-    <t>PSI presentation_2021.pdf</t>
-  </si>
-  <si>
-    <t>16.06.2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helle Lynggaard </t>
-  </si>
-  <si>
-    <t>Non-inferiority and the estimand framework</t>
-  </si>
-  <si>
-    <t>How the estimand framework affects choice of non-inferiority margin</t>
-  </si>
-  <si>
-    <t>19.06.24_11.00-12.30_Helle_Lynggaard.pdf</t>
-  </si>
-  <si>
-    <t>19.06.24_11.00-12.30_David_Wright.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tobias Mütze </t>
-  </si>
-  <si>
-    <t>Kit Roes</t>
-  </si>
-  <si>
-    <t>Chair EMA MWP</t>
-  </si>
-  <si>
-    <t>Florian Lasch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khadija Rantell </t>
-  </si>
-  <si>
-    <t>EIWG_Clinical_Pharmacology_PSI_poster_02June2022_handout.pdf</t>
-  </si>
-  <si>
-    <t>12.06.23_13.30-15.00_1_ICH E9(R1)_impacts_beyond_Bioequivalence_Sue_Helle.pdf</t>
-  </si>
-  <si>
-    <t>2024 PSI Annual Conference - Talks</t>
-  </si>
-  <si>
-    <t>2024 PSI Annual Conference - Panel</t>
-  </si>
-  <si>
-    <t>17.06.2024</t>
-  </si>
-  <si>
-    <t>ICH E9(R1) Implementation in Study Protocols - Speaker 1</t>
-  </si>
-  <si>
-    <t>ICH E9(R1) Implementation in Study Protocols - Speaker 2</t>
-  </si>
-  <si>
-    <t>Does it Make Sense to Apply the Estimand Framework to Clinical Pharmacology Trials? - Speaker 1</t>
-  </si>
-  <si>
-    <t>Does it Make Sense to Apply the Estimand Framework to Clinical Pharmacology Trials? - Speaker 2</t>
-  </si>
-  <si>
-    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 2</t>
-  </si>
-  <si>
-    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 1</t>
-  </si>
-  <si>
-    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 3</t>
-  </si>
-  <si>
-    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 4</t>
-  </si>
-  <si>
-    <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 5</t>
-  </si>
-  <si>
     <t>Estimands in non-inferiority trials: challenges in implementation panel discussion - Panelist 6</t>
   </si>
   <si>
-    <t>EIWG-Intercurrent-Events-Poster-Clean.pdf</t>
-  </si>
-  <si>
-    <t>Vivian Lanius</t>
-  </si>
-  <si>
-    <t>Bayer AG</t>
-  </si>
-  <si>
-    <t>Realizing the benefits of estimands when reporting and communicating study results – some recommendations</t>
-  </si>
-  <si>
-    <t>Poster_EFSPI_EIWG_reporting_2024_final.pdf</t>
-  </si>
-  <si>
-    <t>non-inferiority _poster_final.pdf</t>
-  </si>
-  <si>
-    <t>Considerations when Selecting Strategies for Intercurrent Events in Non-inferiority Trials</t>
-  </si>
-  <si>
     <t>12.06.2024</t>
   </si>
   <si>
+    <t xml:space="preserve"> 2024 NordicEpi  Annual Conference</t>
+  </si>
+  <si>
+    <t>Copenhagen</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>Talk</t>
+  </si>
+  <si>
+    <t>Lotte Husemoen</t>
+  </si>
+  <si>
+    <t>The ICH E9(R1) Estimands Framework in the context of Real-World Data and Observational Studies</t>
+  </si>
+  <si>
     <t>24.08.2024</t>
   </si>
   <si>
+    <t xml:space="preserve"> 2024 ISPE Annual Conference</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>(ENCORE) The ICH E9(R1) Estimands Framework in the context of Real-World Data and Observational Studies</t>
+  </si>
+  <si>
+    <t>01.10.2024</t>
+  </si>
+  <si>
+    <t>2024 DSFE Annual Conference</t>
+  </si>
+  <si>
+    <t>Nyborg</t>
+  </si>
+  <si>
+    <t>Poster (encore)</t>
+  </si>
+  <si>
     <t>14.11.2023</t>
   </si>
   <si>
-    <t xml:space="preserve"> 2024 NordicEpi  Annual Conference</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2024 ISPE Annual Conference</t>
-  </si>
-  <si>
-    <t>2024 DSFE Annual Conference</t>
-  </si>
-  <si>
     <t>2023 ISPOR Annual European conference</t>
   </si>
   <si>
-    <t>Copenhagen</t>
-  </si>
-  <si>
-    <t>Berlin</t>
-  </si>
-  <si>
-    <t>Nyborg</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>Talk</t>
-  </si>
-  <si>
-    <t>Poster (encore)</t>
-  </si>
-  <si>
-    <t>Lotte Husemoen</t>
-  </si>
-  <si>
     <t>Pepa Polavieja/Antonia Morga</t>
   </si>
   <si>
     <t>Novo Nordisk/Astellas</t>
   </si>
   <si>
-    <t>The ICH E9(R1) Estimands Framework in the context of Real-World Data and Observational Studies</t>
-  </si>
-  <si>
-    <t>(ENCORE) The ICH E9(R1) Estimands Framework in the context of Real-World Data and Observational Studies</t>
-  </si>
-  <si>
     <t>Estimands in Health Technology Assessments: methodological considerations and recommendations</t>
   </si>
   <si>
     <t>The ICH E9(R1) Addendum in the context of Health Technology Assessments: methodological considerations and recommendations -  Speaker 3</t>
   </si>
   <si>
-    <t>Denmark</t>
-  </si>
-  <si>
-    <t>01.10.2024</t>
+    <t>16.06.2026</t>
+  </si>
+  <si>
+    <t>2026 PSI Annual Conference</t>
+  </si>
+  <si>
+    <t>Belfast</t>
+  </si>
+  <si>
+    <t>Chun-Hang Tang / Shuying Yang</t>
+  </si>
+  <si>
+    <t>Astellas/GSK</t>
+  </si>
+  <si>
+    <t>Applying the Estimand Framework to Dose-Ranging Trials: A Case Study</t>
+  </si>
+  <si>
+    <t>psi_2026_estimand_dose_ranging_poster.pdf</t>
+  </si>
+  <si>
+    <t>Applying the Estimand Framework to Dose-Ranging Trials: A Case Study Supplementary material</t>
+  </si>
+  <si>
+    <t>Applying the estimand framework to dose ranging trials supplementary material.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -510,8 +537,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="2" xr:uid="{B95AF0D5-A763-4D8C-87A5-63DF3E94DFFF}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -790,29 +817,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P29"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="13.81640625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="23.6328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="27.6328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.08984375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="10.54296875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.08984375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="8.36328125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.26953125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.453125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="6.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.54296875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="15.81640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.81640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="14.54296875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="72.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.08984375" style="1"/>
+    <col min="1" max="1" width="13.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5703125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.85546875" style="2" customWidth="1"/>
+    <col min="15" max="15" width="73.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="72.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -862,24 +889,24 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="43.5">
       <c r="A2" s="4" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>22</v>
@@ -891,30 +918,30 @@
         <v>23</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="57.95">
       <c r="A3" s="4" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>22</v>
@@ -923,65 +950,65 @@
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="57.95">
       <c r="A4" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="K4" s="1">
         <v>1</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="87">
+      <c r="A5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="O4" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="87" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="E5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>22</v>
@@ -993,30 +1020,30 @@
         <v>23</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="57.95">
       <c r="A6" s="4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>22</v>
@@ -1025,33 +1052,33 @@
         <v>1</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="57.95">
       <c r="A7" s="4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>22</v>
@@ -1060,33 +1087,33 @@
         <v>2</v>
       </c>
       <c r="L7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="87">
+      <c r="A8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="87" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>22</v>
@@ -1095,33 +1122,33 @@
         <v>3</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="43.5">
       <c r="A9" s="4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>61</v>
@@ -1136,27 +1163,27 @@
         <v>63</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="43.5">
       <c r="A10" s="4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>61</v>
@@ -1165,33 +1192,33 @@
         <v>2</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="57.95">
       <c r="A11" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>61</v>
@@ -1200,33 +1227,33 @@
         <v>1</v>
       </c>
       <c r="L11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="43.5">
+      <c r="A12" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="N11" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="O11" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="F12" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>22</v>
@@ -1235,33 +1262,33 @@
         <v>2</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="72.599999999999994">
       <c r="A13" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>61</v>
@@ -1270,33 +1297,33 @@
         <v>3</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="72.599999999999994">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>61</v>
@@ -1305,33 +1332,33 @@
         <v>4</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="29.1">
       <c r="A15" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>61</v>
@@ -1340,33 +1367,33 @@
         <v>1</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="57.95">
       <c r="A16" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>61</v>
@@ -1375,257 +1402,257 @@
         <v>2</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="72.599999999999994">
       <c r="A17" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K17" s="1">
         <v>1</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="N17" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" ht="72.599999999999994">
       <c r="A18" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K18" s="1">
         <v>2</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="72.599999999999994">
       <c r="A19" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K19" s="1">
         <v>3</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="72.599999999999994">
       <c r="A20" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K20" s="1">
         <v>4</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="72.599999999999994">
       <c r="A21" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K21" s="1">
         <v>5</v>
       </c>
       <c r="L21" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="72.599999999999994">
+      <c r="A22" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="M21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F22" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="K22" s="1">
         <v>6</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>48</v>
+        <v>107</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="72.599999999999994">
       <c r="A23" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="F23" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="K23" s="1">
         <v>1</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N23" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="72.599999999999994">
       <c r="A24" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>119</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>22</v>
@@ -1634,62 +1661,62 @@
         <v>1</v>
       </c>
       <c r="L24" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="M24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N24" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="72.599999999999994">
+      <c r="A25" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="M24" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="N24" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>114</v>
-      </c>
       <c r="D25" s="5" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K25" s="1">
         <v>1</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="N25" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="87">
+      <c r="A26" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" ht="87" x14ac:dyDescent="0.35">
-      <c r="A26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>116</v>
-      </c>
       <c r="E26" s="1" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>22</v>
@@ -1698,45 +1725,109 @@
         <v>1</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N26" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="130.5" x14ac:dyDescent="0.35">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="130.5">
       <c r="A27" s="5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="K27" s="1">
         <v>1</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N27" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="60.75">
+      <c r="A28" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="O28" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="76.5">
+      <c r="A29" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="O29" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>